<commit_message>
Oslo Exchange duplicates accruals fixed and Iceland
</commit_message>
<xml_diff>
--- a/data/obx_xlsx/AKVA.OL.xlsx
+++ b/data/obx_xlsx/AKVA.OL.xlsx
@@ -12992,15 +12992,9 @@
       <c r="F79" s="15"/>
       <c r="G79" s="15"/>
       <c r="H79" s="15"/>
-      <c r="I79" s="14">
-        <v>401.16</v>
-      </c>
-      <c r="J79" s="14">
-        <v>122.17</v>
-      </c>
-      <c r="K79" s="16">
-        <v>29.97</v>
-      </c>
+      <c r="I79" s="14"/>
+      <c r="J79" s="14"/>
+      <c r="K79" s="16"/>
       <c r="L79" s="16">
         <v>57.82</v>
       </c>

</xml_diff>